<commit_message>
updated schedule times ass
</commit_message>
<xml_diff>
--- a/unit-1-sem-2/sem-2-2025.xlsx
+++ b/unit-1-sem-2/sem-2-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f619e97340dcf560/Desktop/repos/hdip/2025/sem-2-calendar/unit-1-sem-2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\CertCompScience\sem-2-calender\unit-1-sem-2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="191" documentId="11_DBE238A9C5A6DCB16A968737DFB27B2D608E2DA0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7EE36F8-B030-4F68-9650-86EE816EA606}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B247A43F-1A13-4CC1-A80E-B5CB595C6059}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17445" yWindow="-16320" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Export Summary" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,25 @@
     <sheet name="assessment - Table 1-1" sheetId="3" r:id="rId3"/>
     <sheet name="timetable" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="45">
   <si>
     <t>This document was exported from Numbers. Each table was converted to an Excel worksheet. All other objects on each Numbers sheet were placed on separate worksheets. Please be aware that formula calculations may differ in Excel.</t>
   </si>
@@ -88,9 +101,6 @@
     <t>rd</t>
   </si>
   <si>
-    <t xml:space="preserve">Rd	</t>
-  </si>
-  <si>
     <t>Computer Systems &amp; Networks</t>
   </si>
   <si>
@@ -107,15 +117,6 @@
   </si>
   <si>
     <t>Assessment</t>
-  </si>
-  <si>
-    <t>D1a</t>
-  </si>
-  <si>
-    <t>D1b</t>
-  </si>
-  <si>
-    <t>D2</t>
   </si>
   <si>
     <t>timetable</t>
@@ -224,6 +225,33 @@
       <t xml:space="preserve">12:15-2:00 
 </t>
     </r>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>April</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>EASTER</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>E</t>
   </si>
 </sst>
 </file>
@@ -286,11 +314,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color indexed="18"/>
-      <name val="Helvetica Neue Medium"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color indexed="8"/>
       <name val="Helvetica"/>
     </font>
@@ -349,8 +372,13 @@
       <color indexed="8"/>
       <name val="Helvetica"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue Medium"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -389,12 +417,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="21"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor indexed="22"/>
         <bgColor auto="1"/>
       </patternFill>
@@ -411,8 +433,26 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="49">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -569,64 +609,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="17"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top style="thin">
@@ -639,200 +621,6 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="17"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="17"/>
-      </left>
-      <right style="thin">
-        <color indexed="17"/>
-      </right>
-      <top style="thin">
-        <color indexed="17"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="17"/>
-      </left>
-      <right style="thin">
-        <color indexed="17"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="17"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="17"/>
-      </left>
-      <right style="thin">
-        <color indexed="17"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="17"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="17"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="14"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
       <right/>
       <top style="thin">
         <color indexed="13"/>
@@ -1008,13 +796,65 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="14"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right style="thin">
+        <color indexed="13"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="13"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1057,230 +897,215 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="17" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="49" fontId="20" fillId="4" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="13" fillId="11" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="12" fillId="12" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="9" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="9" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="13" fillId="9" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="18" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="18" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1300,47 +1125,53 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="5" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="9" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="19" fillId="10" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="46" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="13" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2573,20 +2404,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:D14"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="13.05" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
-    <col min="2" max="4" width="33.6328125" customWidth="1"/>
+    <col min="2" max="4" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4" ht="0" hidden="1" customHeight="1">
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="84" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-    </row>
-    <row r="7" spans="2:4" ht="17.5">
+      <c r="C3" s="85"/>
+      <c r="D3" s="85"/>
+    </row>
+    <row r="7" spans="2:4" ht="17.399999999999999">
       <c r="B7" s="1" t="s">
         <v>1</v>
       </c>
@@ -2597,14 +2428,14 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.5">
+    <row r="9" spans="2:4" ht="15">
       <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
     </row>
-    <row r="10" spans="2:4" ht="15.5">
+    <row r="10" spans="2:4" ht="15">
       <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
         <v>5</v>
@@ -2613,14 +2444,14 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.5">
+    <row r="11" spans="2:4" ht="15">
       <c r="B11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
     </row>
-    <row r="12" spans="2:4" ht="15.5">
+    <row r="12" spans="2:4" ht="15">
       <c r="B12" s="3"/>
       <c r="C12" s="3" t="s">
         <v>17</v>
@@ -2629,20 +2460,20 @@
         <v>18</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.5">
+    <row r="13" spans="2:4" ht="15">
       <c r="B13" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
     </row>
-    <row r="14" spans="2:4" ht="15.5">
+    <row r="14" spans="2:4" ht="15">
       <c r="B14" s="3"/>
       <c r="C14" s="3" t="s">
         <v>5</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -2664,21 +2495,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultColWidth="16.36328125" defaultRowHeight="20.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="20.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.6328125" style="5" customWidth="1"/>
-    <col min="2" max="2" width="14.453125" style="5" customWidth="1"/>
-    <col min="3" max="9" width="7.6328125" style="5" customWidth="1"/>
-    <col min="10" max="10" width="23.08984375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="16.36328125" style="5" customWidth="1"/>
-    <col min="12" max="16384" width="16.36328125" style="5"/>
+    <col min="1" max="1" width="13.6640625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="5" customWidth="1"/>
+    <col min="3" max="9" width="7.6640625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="23.109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="16.33203125" style="5" customWidth="1"/>
+    <col min="12" max="16384" width="16.33203125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="19.75" customHeight="1">
-      <c r="A1" s="93">
+    <row r="1" spans="1:10" ht="19.8" customHeight="1">
+      <c r="A1" s="88">
         <v>2025</v>
       </c>
-      <c r="B1" s="94"/>
+      <c r="B1" s="89"/>
       <c r="C1" s="6"/>
       <c r="D1" s="7"/>
       <c r="E1" s="7"/>
@@ -2688,11 +2519,11 @@
       <c r="I1" s="7"/>
       <c r="J1" s="8"/>
     </row>
-    <row r="2" spans="1:10" ht="23.75" customHeight="1">
-      <c r="A2" s="91" t="s">
+    <row r="2" spans="1:10" ht="23.7" customHeight="1">
+      <c r="A2" s="86" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="92"/>
+      <c r="B2" s="87"/>
       <c r="C2" s="9" t="s">
         <v>7</v>
       </c>
@@ -2718,548 +2549,674 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="20.75" customHeight="1">
-      <c r="A3" s="12">
-        <v>42248</v>
+    <row r="3" spans="1:10" ht="20.7" customHeight="1">
+      <c r="A3" s="12" t="s">
+        <v>36</v>
       </c>
       <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
-      <c r="I3" s="16"/>
-      <c r="J3" s="17" t="s">
+      <c r="C3" s="59"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60"/>
+      <c r="J3" s="61" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="20" customHeight="1">
-      <c r="A4" s="18"/>
-      <c r="B4" s="19">
+    <row r="4" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A4" s="14"/>
+      <c r="B4" s="55">
         <v>1</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21">
+      <c r="C4" s="62">
+        <v>18</v>
+      </c>
+      <c r="D4" s="63">
+        <v>19</v>
+      </c>
+      <c r="E4" s="62">
+        <f>D4+1</f>
+        <v>20</v>
+      </c>
+      <c r="F4" s="63">
+        <f>E4+1</f>
+        <v>21</v>
+      </c>
+      <c r="G4" s="64">
+        <f>F4+1</f>
+        <v>22</v>
+      </c>
+      <c r="H4" s="62">
+        <f t="shared" ref="H4:I4" si="0">G4+1</f>
+        <v>23</v>
+      </c>
+      <c r="I4" s="62">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="J4" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A5" s="14"/>
+      <c r="B5" s="55">
+        <v>2</v>
+      </c>
+      <c r="C5" s="62">
+        <f>C4+7</f>
+        <v>25</v>
+      </c>
+      <c r="D5" s="63">
+        <f t="shared" ref="D5:I5" si="1">D4+7</f>
+        <v>26</v>
+      </c>
+      <c r="E5" s="62">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+      <c r="F5" s="63">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="G5" s="64">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="H5" s="62">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="I5" s="62">
+        <f t="shared" si="1"/>
+        <v>31</v>
+      </c>
+      <c r="J5" s="66" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A6" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="55">
+        <v>3</v>
+      </c>
+      <c r="C6" s="62">
         <v>1</v>
       </c>
-      <c r="E4" s="22">
+      <c r="D6" s="63">
+        <f>C6+1</f>
         <v>2</v>
       </c>
-      <c r="F4" s="21">
+      <c r="E6" s="62">
+        <f t="shared" ref="E6:I6" si="2">D6+1</f>
         <v>3</v>
       </c>
-      <c r="G4" s="23">
+      <c r="F6" s="63">
+        <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="H4" s="24">
+      <c r="G6" s="64">
+        <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="I4" s="24">
+      <c r="H6" s="62">
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="I6" s="62">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="J6" s="65" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="20" customHeight="1">
-      <c r="A5" s="18"/>
-      <c r="B5" s="19">
+    <row r="7" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A7" s="15"/>
+      <c r="B7" s="5">
+        <v>4</v>
+      </c>
+      <c r="C7" s="62">
+        <f>I6+1</f>
+        <v>8</v>
+      </c>
+      <c r="D7" s="63">
+        <f>C7+1</f>
+        <v>9</v>
+      </c>
+      <c r="E7" s="62">
+        <f t="shared" ref="E7:I7" si="3">D7+1</f>
+        <v>10</v>
+      </c>
+      <c r="F7" s="63">
+        <f t="shared" si="3"/>
+        <v>11</v>
+      </c>
+      <c r="G7" s="64">
+        <f t="shared" si="3"/>
+        <v>12</v>
+      </c>
+      <c r="H7" s="62">
+        <f t="shared" si="3"/>
+        <v>13</v>
+      </c>
+      <c r="I7" s="62">
+        <f t="shared" si="3"/>
+        <v>14</v>
+      </c>
+      <c r="J7" s="67"/>
+    </row>
+    <row r="8" spans="1:10" ht="19.95" customHeight="1">
+      <c r="B8" s="56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="62">
+        <f>C7+7</f>
+        <v>15</v>
+      </c>
+      <c r="D8" s="63">
+        <f t="shared" ref="D8:I9" si="4">D7+7</f>
+        <v>16</v>
+      </c>
+      <c r="E8" s="62">
+        <f t="shared" si="4"/>
+        <v>17</v>
+      </c>
+      <c r="F8" s="63">
+        <f t="shared" si="4"/>
+        <v>18</v>
+      </c>
+      <c r="G8" s="64">
+        <f t="shared" si="4"/>
+        <v>19</v>
+      </c>
+      <c r="H8" s="62">
+        <f t="shared" si="4"/>
+        <v>20</v>
+      </c>
+      <c r="I8" s="62">
+        <f t="shared" si="4"/>
+        <v>21</v>
+      </c>
+      <c r="J8" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A9" s="14"/>
+      <c r="B9" s="55">
+        <v>5</v>
+      </c>
+      <c r="C9" s="62">
+        <f>C8+7</f>
+        <v>22</v>
+      </c>
+      <c r="D9" s="63">
+        <f t="shared" si="4"/>
+        <v>23</v>
+      </c>
+      <c r="E9" s="62">
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="F9" s="63">
+        <f t="shared" si="4"/>
+        <v>25</v>
+      </c>
+      <c r="G9" s="64">
+        <f t="shared" si="4"/>
+        <v>26</v>
+      </c>
+      <c r="H9" s="62">
+        <f t="shared" si="4"/>
+        <v>27</v>
+      </c>
+      <c r="I9" s="62">
+        <f t="shared" si="4"/>
+        <v>28</v>
+      </c>
+      <c r="J9" s="66" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A10" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="55">
+        <v>6</v>
+      </c>
+      <c r="C10" s="62">
+        <v>1</v>
+      </c>
+      <c r="D10" s="63">
+        <f>C10+1</f>
         <v>2</v>
       </c>
-      <c r="C5" s="26">
+      <c r="E10" s="62">
+        <f t="shared" ref="E10:I10" si="5">D10+1</f>
+        <v>3</v>
+      </c>
+      <c r="F10" s="63">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="G10" s="64">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="H10" s="62">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="I10" s="62">
+        <f t="shared" si="5"/>
         <v>7</v>
       </c>
-      <c r="D5" s="27">
+      <c r="J10" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A11" s="15"/>
+      <c r="B11" s="56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="62">
+        <f>C10+7</f>
         <v>8</v>
       </c>
-      <c r="E5" s="28">
+      <c r="D11" s="63">
+        <f t="shared" ref="D11:I14" si="6">D10+7</f>
         <v>9</v>
       </c>
-      <c r="F5" s="27">
+      <c r="E11" s="62">
+        <f t="shared" si="6"/>
         <v>10</v>
       </c>
-      <c r="G5" s="23">
+      <c r="F11" s="63">
+        <f t="shared" si="6"/>
         <v>11</v>
       </c>
-      <c r="H5" s="29">
+      <c r="G11" s="64">
+        <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="I5" s="29">
+      <c r="H11" s="62">
+        <f t="shared" si="6"/>
         <v>13</v>
       </c>
-      <c r="J5" s="30" t="s">
+      <c r="I11" s="62">
+        <f t="shared" si="6"/>
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="20" customHeight="1">
-      <c r="A6" s="18"/>
-      <c r="B6" s="19">
+      <c r="J11" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="19.95" customHeight="1">
+      <c r="B12" s="5">
+        <v>7</v>
+      </c>
+      <c r="C12" s="62">
+        <f>C11+7</f>
+        <v>15</v>
+      </c>
+      <c r="D12" s="63">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="E12" s="62">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="F12" s="63">
+        <f t="shared" si="6"/>
+        <v>18</v>
+      </c>
+      <c r="G12" s="64">
+        <f t="shared" si="6"/>
+        <v>19</v>
+      </c>
+      <c r="H12" s="62">
+        <f t="shared" si="6"/>
+        <v>20</v>
+      </c>
+      <c r="I12" s="62">
+        <f t="shared" si="6"/>
+        <v>21</v>
+      </c>
+      <c r="J12" s="68"/>
+    </row>
+    <row r="13" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A13" s="14"/>
+      <c r="B13" s="55">
+        <v>8</v>
+      </c>
+      <c r="C13" s="62">
+        <f>C12+7</f>
+        <v>22</v>
+      </c>
+      <c r="D13" s="63">
+        <f t="shared" si="6"/>
+        <v>23</v>
+      </c>
+      <c r="E13" s="62">
+        <f t="shared" si="6"/>
+        <v>24</v>
+      </c>
+      <c r="F13" s="63">
+        <f t="shared" si="6"/>
+        <v>25</v>
+      </c>
+      <c r="G13" s="64">
+        <f t="shared" si="6"/>
+        <v>26</v>
+      </c>
+      <c r="H13" s="62">
+        <f t="shared" si="6"/>
+        <v>27</v>
+      </c>
+      <c r="I13" s="62">
+        <f t="shared" si="6"/>
+        <v>28</v>
+      </c>
+      <c r="J13" s="66" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A14" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="62">
+        <f>C13+7</f>
+        <v>29</v>
+      </c>
+      <c r="D14" s="63">
+        <f t="shared" si="6"/>
+        <v>30</v>
+      </c>
+      <c r="E14" s="62">
+        <f t="shared" si="6"/>
+        <v>31</v>
+      </c>
+      <c r="F14" s="63">
+        <v>1</v>
+      </c>
+      <c r="G14" s="64">
+        <f>F14+1</f>
+        <v>2</v>
+      </c>
+      <c r="H14" s="62">
+        <f t="shared" ref="H14:I14" si="7">G14+1</f>
         <v>3</v>
       </c>
-      <c r="C6" s="20">
+      <c r="I14" s="62">
+        <f t="shared" si="7"/>
+        <v>4</v>
+      </c>
+      <c r="J14" s="65" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="27">
+    </row>
+    <row r="15" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A15" s="15"/>
+      <c r="B15" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="62">
+        <f>I14+1</f>
+        <v>5</v>
+      </c>
+      <c r="D15" s="63">
+        <f>C15+1</f>
+        <v>6</v>
+      </c>
+      <c r="E15" s="62">
+        <f t="shared" ref="E15:I15" si="8">D15+1</f>
+        <v>7</v>
+      </c>
+      <c r="F15" s="63">
+        <f t="shared" si="8"/>
+        <v>8</v>
+      </c>
+      <c r="G15" s="64">
+        <f t="shared" si="8"/>
+        <v>9</v>
+      </c>
+      <c r="H15" s="62">
+        <f t="shared" si="8"/>
+        <v>10</v>
+      </c>
+      <c r="I15" s="62">
+        <f t="shared" si="8"/>
+        <v>11</v>
+      </c>
+      <c r="J15" s="67"/>
+    </row>
+    <row r="16" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A16" s="15"/>
+      <c r="B16" s="55">
+        <v>9</v>
+      </c>
+      <c r="C16" s="62">
+        <f>C15+7</f>
+        <v>12</v>
+      </c>
+      <c r="D16" s="63">
+        <f t="shared" ref="D16:I18" si="9">D15+7</f>
+        <v>13</v>
+      </c>
+      <c r="E16" s="62">
+        <f t="shared" si="9"/>
+        <v>14</v>
+      </c>
+      <c r="F16" s="63">
+        <f t="shared" si="9"/>
         <v>15</v>
       </c>
-      <c r="E6" s="22">
+      <c r="G16" s="64">
+        <f t="shared" si="9"/>
         <v>16</v>
       </c>
-      <c r="F6" s="27">
+      <c r="H16" s="62">
+        <f t="shared" si="9"/>
         <v>17</v>
       </c>
-      <c r="G6" s="23">
+      <c r="I16" s="62">
+        <f t="shared" si="9"/>
         <v>18</v>
       </c>
-      <c r="H6" s="24">
+      <c r="J16" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="19.95" customHeight="1">
+      <c r="B17" s="55">
+        <v>10</v>
+      </c>
+      <c r="C17" s="62">
+        <f>C16+7</f>
         <v>19</v>
       </c>
-      <c r="I6" s="24">
+      <c r="D17" s="63">
+        <f t="shared" si="9"/>
         <v>20</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="E17" s="62">
+        <f t="shared" si="9"/>
+        <v>21</v>
+      </c>
+      <c r="F17" s="63">
+        <f t="shared" si="9"/>
+        <v>22</v>
+      </c>
+      <c r="G17" s="64">
+        <f t="shared" si="9"/>
+        <v>23</v>
+      </c>
+      <c r="H17" s="62">
+        <f t="shared" si="9"/>
+        <v>24</v>
+      </c>
+      <c r="I17" s="62">
+        <f t="shared" si="9"/>
+        <v>25</v>
+      </c>
+      <c r="J17" s="66" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="20" customHeight="1">
-      <c r="A7" s="31"/>
-      <c r="B7" s="32" t="s">
+    <row r="18" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A18" s="17"/>
+      <c r="B18" s="55">
+        <v>11</v>
+      </c>
+      <c r="C18" s="62">
+        <f>C17+7</f>
+        <v>26</v>
+      </c>
+      <c r="D18" s="63">
+        <f t="shared" si="9"/>
+        <v>27</v>
+      </c>
+      <c r="E18" s="62">
+        <f t="shared" si="9"/>
+        <v>28</v>
+      </c>
+      <c r="F18" s="63">
+        <f t="shared" si="9"/>
+        <v>29</v>
+      </c>
+      <c r="G18" s="64">
+        <f>G17+7</f>
+        <v>30</v>
+      </c>
+      <c r="H18" s="62">
+        <v>1</v>
+      </c>
+      <c r="I18" s="62">
+        <v>2</v>
+      </c>
+      <c r="J18" s="65" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A19" s="105" t="s">
+        <v>40</v>
+      </c>
+      <c r="B19" s="55">
+        <v>12</v>
+      </c>
+      <c r="C19" s="69">
+        <f>I18+1</f>
+        <v>3</v>
+      </c>
+      <c r="D19" s="70">
+        <f>C19+1</f>
+        <v>4</v>
+      </c>
+      <c r="E19" s="69">
+        <f t="shared" ref="E19:I19" si="10">D19+1</f>
+        <v>5</v>
+      </c>
+      <c r="F19" s="70">
+        <f t="shared" si="10"/>
+        <v>6</v>
+      </c>
+      <c r="G19" s="64">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="H19" s="69">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+      <c r="I19" s="69">
+        <f t="shared" si="10"/>
+        <v>9</v>
+      </c>
+      <c r="J19" s="66" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="19.95" customHeight="1">
+      <c r="A20" s="15"/>
+      <c r="B20" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="33">
+      <c r="C20" s="69">
+        <f>C19+7</f>
+        <v>10</v>
+      </c>
+      <c r="D20" s="70">
+        <f t="shared" ref="D20:I21" si="11">D19+7</f>
+        <v>11</v>
+      </c>
+      <c r="E20" s="69">
+        <f t="shared" si="11"/>
+        <v>12</v>
+      </c>
+      <c r="F20" s="70">
+        <f t="shared" si="11"/>
+        <v>13</v>
+      </c>
+      <c r="G20" s="64">
+        <f t="shared" si="11"/>
+        <v>14</v>
+      </c>
+      <c r="H20" s="69">
+        <f t="shared" si="11"/>
+        <v>15</v>
+      </c>
+      <c r="I20" s="69">
+        <f t="shared" si="11"/>
+        <v>16</v>
+      </c>
+      <c r="J20" s="65"/>
+    </row>
+    <row r="21" spans="1:10" ht="19.8" customHeight="1">
+      <c r="B21" s="58" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="69">
+        <f>C20+7</f>
+        <v>17</v>
+      </c>
+      <c r="D21" s="70">
+        <f t="shared" si="11"/>
+        <v>18</v>
+      </c>
+      <c r="E21" s="69">
+        <f t="shared" si="11"/>
+        <v>19</v>
+      </c>
+      <c r="F21" s="70">
+        <f t="shared" si="11"/>
+        <v>20</v>
+      </c>
+      <c r="G21" s="64">
+        <f t="shared" si="11"/>
         <v>21</v>
       </c>
-      <c r="D7" s="34">
+      <c r="H21" s="69">
+        <f t="shared" si="11"/>
         <v>22</v>
       </c>
-      <c r="E7" s="34">
+      <c r="I21" s="69">
+        <f t="shared" si="11"/>
         <v>23</v>
       </c>
-      <c r="F7" s="34">
-        <v>24</v>
-      </c>
-      <c r="G7" s="35">
-        <v>25</v>
-      </c>
-      <c r="H7" s="36">
-        <v>26</v>
-      </c>
-      <c r="I7" s="36">
-        <v>27</v>
-      </c>
-      <c r="J7" s="37"/>
-    </row>
-    <row r="8" spans="1:10" ht="20" customHeight="1">
-      <c r="A8" s="38">
-        <v>43374</v>
-      </c>
-      <c r="B8" s="19">
-        <v>4</v>
-      </c>
-      <c r="C8" s="20">
-        <v>28</v>
-      </c>
-      <c r="D8" s="27">
-        <v>29</v>
-      </c>
-      <c r="E8" s="22">
-        <v>30</v>
-      </c>
-      <c r="F8" s="27">
-        <v>1</v>
-      </c>
-      <c r="G8" s="23">
-        <v>2</v>
-      </c>
-      <c r="H8" s="24">
-        <v>3</v>
-      </c>
-      <c r="I8" s="24">
-        <v>4</v>
-      </c>
-      <c r="J8" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="20" customHeight="1">
-      <c r="A9" s="18"/>
-      <c r="B9" s="19">
-        <v>5</v>
-      </c>
-      <c r="C9" s="26">
-        <v>5</v>
-      </c>
-      <c r="D9" s="27">
-        <v>6</v>
-      </c>
-      <c r="E9" s="28">
-        <v>7</v>
-      </c>
-      <c r="F9" s="27">
-        <v>8</v>
-      </c>
-      <c r="G9" s="23">
-        <v>9</v>
-      </c>
-      <c r="H9" s="29">
-        <v>10</v>
-      </c>
-      <c r="I9" s="29">
-        <v>11</v>
-      </c>
-      <c r="J9" s="30" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="20" customHeight="1">
-      <c r="A10" s="18"/>
-      <c r="B10" s="19">
-        <v>6</v>
-      </c>
-      <c r="C10" s="20">
-        <v>12</v>
-      </c>
-      <c r="D10" s="27">
-        <v>13</v>
-      </c>
-      <c r="E10" s="22">
-        <v>14</v>
-      </c>
-      <c r="F10" s="27">
-        <v>15</v>
-      </c>
-      <c r="G10" s="23">
-        <v>16</v>
-      </c>
-      <c r="H10" s="24">
-        <v>17</v>
-      </c>
-      <c r="I10" s="24">
-        <v>18</v>
-      </c>
-      <c r="J10" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="20" customHeight="1">
-      <c r="A11" s="31"/>
-      <c r="B11" s="19">
-        <v>7</v>
-      </c>
-      <c r="C11" s="20">
-        <v>19</v>
-      </c>
-      <c r="D11" s="27">
-        <v>20</v>
-      </c>
-      <c r="E11" s="22">
-        <v>21</v>
-      </c>
-      <c r="F11" s="27">
-        <v>22</v>
-      </c>
-      <c r="G11" s="23">
-        <v>23</v>
-      </c>
-      <c r="H11" s="24">
-        <v>24</v>
-      </c>
-      <c r="I11" s="24">
-        <v>25</v>
-      </c>
-      <c r="J11" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="20" customHeight="1">
-      <c r="A12" s="38">
-        <v>43405</v>
-      </c>
-      <c r="B12" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="33">
-        <v>26</v>
-      </c>
-      <c r="D12" s="34">
-        <v>27</v>
-      </c>
-      <c r="E12" s="34">
-        <v>28</v>
-      </c>
-      <c r="F12" s="34">
-        <v>29</v>
-      </c>
-      <c r="G12" s="35">
-        <v>30</v>
-      </c>
-      <c r="H12" s="36">
-        <v>31</v>
-      </c>
-      <c r="I12" s="36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="20" customHeight="1">
-      <c r="A13" s="18"/>
-      <c r="B13" s="19">
-        <v>8</v>
-      </c>
-      <c r="C13" s="26">
-        <v>2</v>
-      </c>
-      <c r="D13" s="27">
-        <v>3</v>
-      </c>
-      <c r="E13" s="28">
-        <v>4</v>
-      </c>
-      <c r="F13" s="27">
-        <v>5</v>
-      </c>
-      <c r="G13" s="23">
-        <v>6</v>
-      </c>
-      <c r="H13" s="29">
-        <v>7</v>
-      </c>
-      <c r="I13" s="29">
-        <v>8</v>
-      </c>
-      <c r="J13" s="30" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="20" customHeight="1">
-      <c r="A14" s="18"/>
-      <c r="B14" s="39">
-        <v>9</v>
-      </c>
-      <c r="C14" s="20">
-        <v>9</v>
-      </c>
-      <c r="D14" s="27">
-        <v>10</v>
-      </c>
-      <c r="E14" s="22">
-        <v>11</v>
-      </c>
-      <c r="F14" s="27">
-        <v>12</v>
-      </c>
-      <c r="G14" s="23">
-        <v>13</v>
-      </c>
-      <c r="H14" s="24">
-        <v>14</v>
-      </c>
-      <c r="I14" s="24">
-        <v>15</v>
-      </c>
-      <c r="J14" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="20" customHeight="1">
-      <c r="A15" s="31"/>
-      <c r="B15" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="33">
-        <v>16</v>
-      </c>
-      <c r="D15" s="34">
-        <v>17</v>
-      </c>
-      <c r="E15" s="34">
-        <v>18</v>
-      </c>
-      <c r="F15" s="34">
-        <v>19</v>
-      </c>
-      <c r="G15" s="35">
-        <v>20</v>
-      </c>
-      <c r="H15" s="36">
-        <v>21</v>
-      </c>
-      <c r="I15" s="36">
-        <v>22</v>
-      </c>
-      <c r="J15" s="37"/>
-    </row>
-    <row r="16" spans="1:10" ht="20" customHeight="1">
-      <c r="A16" s="31"/>
-      <c r="B16" s="19">
-        <v>10</v>
-      </c>
-      <c r="C16" s="20">
-        <v>23</v>
-      </c>
-      <c r="D16" s="27">
-        <v>24</v>
-      </c>
-      <c r="E16" s="22">
-        <v>25</v>
-      </c>
-      <c r="F16" s="27">
-        <v>26</v>
-      </c>
-      <c r="G16" s="23">
-        <v>27</v>
-      </c>
-      <c r="H16" s="24">
-        <v>28</v>
-      </c>
-      <c r="I16" s="24">
-        <v>29</v>
-      </c>
-      <c r="J16" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="20" customHeight="1">
-      <c r="A17" s="38">
-        <v>43435</v>
-      </c>
-      <c r="B17" s="19">
-        <v>11</v>
-      </c>
-      <c r="C17" s="26">
-        <v>30</v>
-      </c>
-      <c r="D17" s="27">
-        <v>1</v>
-      </c>
-      <c r="E17" s="28">
-        <v>2</v>
-      </c>
-      <c r="F17" s="27">
-        <v>3</v>
-      </c>
-      <c r="G17" s="23">
-        <v>4</v>
-      </c>
-      <c r="H17" s="29">
-        <v>5</v>
-      </c>
-      <c r="I17" s="29">
-        <v>6</v>
-      </c>
-      <c r="J17" s="30" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="20" customHeight="1">
-      <c r="A18" s="40"/>
-      <c r="B18" s="19">
-        <v>12</v>
-      </c>
-      <c r="C18" s="20">
-        <v>7</v>
-      </c>
-      <c r="D18" s="41">
-        <v>8</v>
-      </c>
-      <c r="E18" s="22">
-        <v>9</v>
-      </c>
-      <c r="F18" s="41">
-        <v>10</v>
-      </c>
-      <c r="G18" s="23">
-        <v>11</v>
-      </c>
-      <c r="H18" s="24">
-        <v>12</v>
-      </c>
-      <c r="I18" s="24">
-        <v>13</v>
-      </c>
-      <c r="J18" s="25" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="20" customHeight="1">
-      <c r="A19" s="40"/>
-      <c r="B19" s="42"/>
-      <c r="C19" s="43">
-        <v>14</v>
-      </c>
-      <c r="D19" s="44">
-        <v>15</v>
-      </c>
-      <c r="E19" s="45">
-        <v>16</v>
-      </c>
-      <c r="F19" s="44">
-        <v>17</v>
-      </c>
-      <c r="G19" s="45">
-        <v>18</v>
-      </c>
-      <c r="H19" s="45">
-        <v>19</v>
-      </c>
-      <c r="I19" s="45">
-        <v>20</v>
-      </c>
-      <c r="J19" s="37"/>
-    </row>
-    <row r="20" spans="1:10" ht="20" customHeight="1">
-      <c r="A20" s="31"/>
-      <c r="B20" s="42"/>
-      <c r="C20" s="46">
-        <v>21</v>
-      </c>
-      <c r="D20" s="47">
-        <v>22</v>
-      </c>
-      <c r="E20" s="47">
-        <v>23</v>
-      </c>
-      <c r="F20" s="47">
-        <v>24</v>
-      </c>
-      <c r="G20" s="47">
-        <v>25</v>
-      </c>
-      <c r="H20" s="47">
-        <v>26</v>
-      </c>
-      <c r="I20" s="47">
-        <v>27</v>
-      </c>
-      <c r="J20" s="48"/>
-    </row>
-    <row r="21" spans="1:10" ht="19.75" customHeight="1">
-      <c r="A21" s="49">
-        <v>43101</v>
-      </c>
-      <c r="B21" s="50"/>
-      <c r="C21" s="51">
-        <v>28</v>
-      </c>
-      <c r="D21" s="52">
-        <v>29</v>
-      </c>
-      <c r="E21" s="52">
-        <v>30</v>
-      </c>
-      <c r="F21" s="52">
-        <v>31</v>
-      </c>
-      <c r="G21" s="52">
-        <v>1</v>
-      </c>
-      <c r="H21" s="52">
-        <v>2</v>
-      </c>
-      <c r="I21" s="52">
-        <v>3</v>
-      </c>
-      <c r="J21" s="53"/>
+      <c r="J21" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3271,6 +3228,9 @@
   <headerFooter>
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
+  <ignoredErrors>
+    <ignoredError sqref="E5" formula="1"/>
+  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -3280,472 +3240,482 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC12"/>
-  <sheetFormatPr defaultColWidth="16.36328125" defaultRowHeight="18" customHeight="1"/>
+  <dimension ref="A1:AD12"/>
+  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="18" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="18.26953125" style="54" customWidth="1"/>
-    <col min="2" max="5" width="4.08984375" style="54" customWidth="1"/>
-    <col min="6" max="6" width="1.6328125" style="54" customWidth="1"/>
-    <col min="7" max="7" width="4.08984375" style="54" customWidth="1"/>
-    <col min="8" max="8" width="1.6328125" style="54" customWidth="1"/>
-    <col min="9" max="11" width="4.08984375" style="54" customWidth="1"/>
-    <col min="12" max="12" width="4" style="54" customWidth="1"/>
-    <col min="13" max="13" width="1.453125" style="54" customWidth="1"/>
-    <col min="14" max="14" width="3.453125" style="54" customWidth="1"/>
-    <col min="15" max="15" width="1.7265625" style="54" customWidth="1"/>
-    <col min="16" max="17" width="4.08984375" style="54" customWidth="1"/>
-    <col min="18" max="18" width="1.81640625" style="54" customWidth="1"/>
-    <col min="19" max="19" width="2.81640625" style="54" customWidth="1"/>
-    <col min="20" max="20" width="1.7265625" style="54" customWidth="1"/>
-    <col min="21" max="21" width="4.453125" style="54" customWidth="1"/>
-    <col min="22" max="23" width="4.08984375" style="54" customWidth="1"/>
-    <col min="24" max="24" width="1.6328125" style="54" customWidth="1"/>
-    <col min="25" max="27" width="4.08984375" style="54" customWidth="1"/>
-    <col min="28" max="28" width="4.1796875" style="54" customWidth="1"/>
-    <col min="29" max="29" width="3.6328125" style="54" customWidth="1"/>
-    <col min="30" max="30" width="16.36328125" style="54" customWidth="1"/>
-    <col min="31" max="16384" width="16.36328125" style="54"/>
+    <col min="1" max="1" width="18.21875" style="18" customWidth="1"/>
+    <col min="2" max="6" width="4.109375" style="18" customWidth="1"/>
+    <col min="7" max="7" width="1.6640625" style="18" customWidth="1"/>
+    <col min="8" max="8" width="4.109375" style="18" customWidth="1"/>
+    <col min="9" max="9" width="1" style="18" customWidth="1"/>
+    <col min="10" max="11" width="4.109375" style="18" customWidth="1"/>
+    <col min="12" max="12" width="1" style="77" customWidth="1"/>
+    <col min="13" max="13" width="4" style="18" customWidth="1"/>
+    <col min="14" max="14" width="1.44140625" style="18" customWidth="1"/>
+    <col min="15" max="15" width="3.44140625" style="18" customWidth="1"/>
+    <col min="16" max="16" width="4.109375" style="18" customWidth="1"/>
+    <col min="17" max="17" width="1.33203125" style="18" customWidth="1"/>
+    <col min="18" max="18" width="4.109375" style="18" customWidth="1"/>
+    <col min="19" max="19" width="3.33203125" style="18" customWidth="1"/>
+    <col min="20" max="20" width="1.77734375" style="18" customWidth="1"/>
+    <col min="21" max="21" width="4.44140625" style="18" customWidth="1"/>
+    <col min="22" max="24" width="4.109375" style="18" customWidth="1"/>
+    <col min="25" max="25" width="1.6640625" style="18" customWidth="1"/>
+    <col min="26" max="28" width="4.109375" style="18" customWidth="1"/>
+    <col min="29" max="29" width="4.21875" style="18" customWidth="1"/>
+    <col min="30" max="30" width="3.6640625" style="18" customWidth="1"/>
+    <col min="31" max="31" width="16.33203125" style="18" customWidth="1"/>
+    <col min="32" max="16384" width="16.33203125" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="20" customHeight="1">
-      <c r="A1" s="55"/>
-      <c r="B1" s="56"/>
-      <c r="C1" s="96">
-        <v>43709</v>
-      </c>
-      <c r="D1" s="95"/>
-      <c r="E1" s="95"/>
-      <c r="F1" s="96">
-        <v>43739</v>
-      </c>
-      <c r="G1" s="95"/>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="96">
-        <v>43770</v>
-      </c>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="95"/>
-      <c r="O1" s="95"/>
-      <c r="P1" s="96">
-        <v>43800</v>
-      </c>
-      <c r="Q1" s="95"/>
-      <c r="R1" s="95"/>
-      <c r="S1" s="95"/>
-      <c r="T1" s="95"/>
-      <c r="U1" s="95"/>
-      <c r="V1" s="95"/>
-      <c r="W1" s="95"/>
-      <c r="X1" s="95"/>
-      <c r="Y1" s="95"/>
-      <c r="Z1" s="95"/>
-      <c r="AA1" s="96">
-        <v>43466</v>
-      </c>
-      <c r="AB1" s="95"/>
-      <c r="AC1" s="95"/>
-    </row>
-    <row r="2" spans="1:29" ht="20" customHeight="1">
-      <c r="A2" s="57" t="s">
+    <row r="1" spans="1:30" ht="19.95" customHeight="1">
+      <c r="A1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="90">
+        <v>46023</v>
+      </c>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="49"/>
+      <c r="J1" s="20"/>
+      <c r="K1" s="90">
+        <v>46082</v>
+      </c>
+      <c r="L1" s="93"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
+      <c r="O1" s="91"/>
+      <c r="P1" s="90">
+        <v>46113</v>
+      </c>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="91"/>
+      <c r="W1" s="94"/>
+      <c r="X1" s="91"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="91"/>
+      <c r="AB1" s="90">
+        <v>46143</v>
+      </c>
+      <c r="AC1" s="91"/>
+      <c r="AD1" s="91"/>
+    </row>
+    <row r="2" spans="1:30" ht="19.95" customHeight="1">
+      <c r="A2" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="55"/>
-      <c r="C2" s="58">
+      <c r="B2" s="19"/>
+      <c r="C2" s="22">
         <v>1</v>
       </c>
-      <c r="D2" s="58">
+      <c r="D2" s="22">
         <v>2</v>
       </c>
-      <c r="E2" s="58">
+      <c r="E2" s="22">
         <v>3</v>
       </c>
-      <c r="F2" s="55"/>
-      <c r="G2" s="59" t="s">
+      <c r="F2" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" s="19"/>
+      <c r="H2" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="H2" s="55"/>
-      <c r="I2" s="58">
-        <v>4</v>
-      </c>
-      <c r="J2" s="58">
+      <c r="I2" s="71"/>
+      <c r="J2" s="22">
         <v>5</v>
       </c>
-      <c r="K2" s="58">
+      <c r="K2" s="22">
         <v>6</v>
       </c>
-      <c r="L2" s="58">
-        <v>7</v>
-      </c>
-      <c r="N2" s="59" t="s">
+      <c r="L2" s="72"/>
+      <c r="M2" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="P2" s="58">
+      <c r="O2" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="P2" s="22">
         <v>8</v>
       </c>
-      <c r="Q2" s="58">
+      <c r="Q2" s="71"/>
+      <c r="R2" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="S2" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="U2" s="22">
         <v>9</v>
       </c>
-      <c r="R2" s="56"/>
-      <c r="S2" s="59" t="s">
+      <c r="V2" s="22">
+        <v>10</v>
+      </c>
+      <c r="W2" s="71">
+        <v>11</v>
+      </c>
+      <c r="X2" s="22">
+        <v>12</v>
+      </c>
+      <c r="Y2" s="19"/>
+      <c r="Z2" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="58">
-        <v>10</v>
-      </c>
-      <c r="V2" s="58">
-        <v>11</v>
-      </c>
-      <c r="W2" s="58">
-        <v>12</v>
-      </c>
-      <c r="X2" s="55"/>
-      <c r="Y2" s="59" t="s">
+      <c r="AA2" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB2" s="92"/>
+      <c r="AC2" s="91"/>
+      <c r="AD2" s="19"/>
+    </row>
+    <row r="3" spans="1:30" ht="10.050000000000001" customHeight="1">
+      <c r="A3" s="24"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="73"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="49"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="25"/>
+      <c r="R3" s="25"/>
+      <c r="S3" s="25"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="25"/>
+      <c r="V3" s="25"/>
+      <c r="W3" s="25"/>
+      <c r="X3" s="25"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="25"/>
+      <c r="AA3" s="25"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="25"/>
+      <c r="AD3" s="19"/>
+    </row>
+    <row r="4" spans="1:30" ht="34.950000000000003" customHeight="1">
+      <c r="A4" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="Z2" s="55"/>
-      <c r="AA2" s="97"/>
-      <c r="AB2" s="95"/>
-      <c r="AC2" s="55"/>
-    </row>
-    <row r="3" spans="1:29" ht="10" customHeight="1">
-      <c r="A3" s="60"/>
-      <c r="B3" s="55"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="61"/>
-      <c r="E3" s="61"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="61"/>
-      <c r="H3" s="55"/>
-      <c r="I3" s="61"/>
-      <c r="J3" s="61"/>
-      <c r="K3" s="61"/>
-      <c r="L3" s="55"/>
-      <c r="M3" s="102"/>
-      <c r="N3" s="55"/>
-      <c r="O3" s="102"/>
-      <c r="P3" s="61"/>
-      <c r="Q3" s="61"/>
-      <c r="R3" s="55"/>
-      <c r="S3" s="61"/>
-      <c r="T3" s="55"/>
-      <c r="U3" s="61"/>
-      <c r="V3" s="61"/>
-      <c r="W3" s="61"/>
-      <c r="X3" s="55"/>
-      <c r="Y3" s="61"/>
-      <c r="Z3" s="61"/>
-      <c r="AA3" s="62"/>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="55"/>
-    </row>
-    <row r="4" spans="1:29" ht="35" customHeight="1">
-      <c r="A4" s="57" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="50"/>
+      <c r="I4" s="80"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="74"/>
+      <c r="M4" s="50"/>
+      <c r="N4" s="52"/>
+      <c r="O4" s="78"/>
+      <c r="P4" s="51"/>
+      <c r="Q4" s="82"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="30"/>
+      <c r="T4" s="29"/>
+      <c r="U4" s="28"/>
+      <c r="V4" s="28"/>
+      <c r="W4" s="28"/>
+      <c r="X4" s="28"/>
+      <c r="Y4" s="29"/>
+      <c r="Z4" s="30"/>
+      <c r="AA4" s="30"/>
+      <c r="AB4" s="30"/>
+      <c r="AC4" s="30"/>
+      <c r="AD4" s="31"/>
+    </row>
+    <row r="5" spans="1:30" ht="10.050000000000001" customHeight="1">
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
+      <c r="K5" s="32"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="49"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="32"/>
+      <c r="S5" s="32"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="32"/>
+      <c r="V5" s="32"/>
+      <c r="W5" s="32"/>
+      <c r="X5" s="32"/>
+      <c r="Y5" s="19"/>
+      <c r="Z5" s="32"/>
+      <c r="AA5" s="32"/>
+      <c r="AB5" s="32"/>
+      <c r="AC5" s="32"/>
+      <c r="AD5" s="19"/>
+    </row>
+    <row r="6" spans="1:30" ht="19.95" customHeight="1">
+      <c r="A6" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="63"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="65"/>
-      <c r="G4" s="66"/>
-      <c r="H4" s="65"/>
-      <c r="I4" s="64"/>
-      <c r="J4" s="64"/>
-      <c r="K4" s="64"/>
-      <c r="L4" s="101"/>
-      <c r="M4" s="105"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="105"/>
-      <c r="P4" s="104"/>
-      <c r="Q4" s="64"/>
-      <c r="R4" s="105"/>
-      <c r="S4" s="66"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="64"/>
-      <c r="V4" s="64"/>
-      <c r="W4" s="64"/>
-      <c r="X4" s="65"/>
-      <c r="Y4" s="66"/>
-      <c r="Z4" s="66"/>
-      <c r="AA4" s="66"/>
-      <c r="AB4" s="66"/>
-      <c r="AC4" s="67"/>
-    </row>
-    <row r="5" spans="1:29" ht="10" customHeight="1">
-      <c r="A5" s="55"/>
-      <c r="B5" s="55"/>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="68"/>
-      <c r="H5" s="55"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="68"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="55"/>
-      <c r="M5" s="102"/>
-      <c r="N5" s="55"/>
-      <c r="O5" s="102"/>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="55"/>
-      <c r="S5" s="68"/>
-      <c r="T5" s="55"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="55"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="68"/>
-      <c r="AA5" s="68"/>
-      <c r="AB5" s="68"/>
-      <c r="AC5" s="55"/>
-    </row>
-    <row r="6" spans="1:29" ht="20" customHeight="1">
-      <c r="A6" s="69" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="79"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="55"/>
-      <c r="C6" s="55"/>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="70"/>
-      <c r="H6" s="70"/>
-      <c r="I6" s="70"/>
-      <c r="J6" s="70"/>
-      <c r="K6" s="71" t="s">
+      <c r="L6" s="83"/>
+      <c r="M6" s="34"/>
+      <c r="N6" s="34"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="34"/>
+      <c r="Q6" s="79"/>
+      <c r="R6" s="34"/>
+      <c r="S6" s="34"/>
+      <c r="T6" s="34"/>
+      <c r="U6" s="34"/>
+      <c r="V6" s="34"/>
+      <c r="W6" s="79"/>
+      <c r="X6" s="34"/>
+      <c r="Y6" s="34"/>
+      <c r="Z6" s="34"/>
+      <c r="AA6" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="70"/>
-      <c r="M6" s="70"/>
-      <c r="N6" s="60"/>
-      <c r="O6" s="55"/>
-      <c r="P6" s="70"/>
-      <c r="Q6" s="70"/>
-      <c r="R6" s="70"/>
-      <c r="S6" s="70"/>
-      <c r="T6" s="70"/>
-      <c r="U6" s="70"/>
-      <c r="V6" s="70"/>
-      <c r="W6" s="70"/>
-      <c r="X6" s="70"/>
-      <c r="Y6" s="70"/>
-      <c r="Z6" s="71" t="s">
+      <c r="AB6" s="24"/>
+      <c r="AC6" s="19"/>
+      <c r="AD6" s="19"/>
+    </row>
+    <row r="7" spans="1:30" ht="19.95" customHeight="1">
+      <c r="A7" s="36"/>
+      <c r="B7" s="19"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="49"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="49"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="49"/>
+      <c r="X7" s="19"/>
+      <c r="Y7" s="19"/>
+      <c r="Z7" s="19"/>
+      <c r="AA7" s="19"/>
+      <c r="AB7" s="19"/>
+      <c r="AC7" s="24"/>
+      <c r="AD7" s="19"/>
+    </row>
+    <row r="8" spans="1:30" ht="10.050000000000001" customHeight="1">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="25"/>
+      <c r="J8" s="25"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="73"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="49"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="25"/>
+      <c r="R8" s="25"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="25"/>
+      <c r="V8" s="25"/>
+      <c r="W8" s="25"/>
+      <c r="X8" s="25"/>
+      <c r="Y8" s="19"/>
+      <c r="Z8" s="25"/>
+      <c r="AA8" s="25"/>
+      <c r="AB8" s="25"/>
+      <c r="AC8" s="25"/>
+      <c r="AD8" s="19"/>
+    </row>
+    <row r="9" spans="1:30" ht="34.950000000000003" customHeight="1">
+      <c r="A9" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="AA6" s="60"/>
-      <c r="AB6" s="55"/>
-      <c r="AC6" s="55"/>
-    </row>
-    <row r="7" spans="1:29" ht="20" customHeight="1">
-      <c r="A7" s="72"/>
-      <c r="B7" s="55"/>
-      <c r="C7" s="55"/>
-      <c r="D7" s="55"/>
-      <c r="E7" s="55"/>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
-      <c r="I7" s="55"/>
-      <c r="J7" s="55"/>
-      <c r="K7" s="55"/>
-      <c r="L7" s="55"/>
-      <c r="M7" s="55"/>
-      <c r="N7" s="55"/>
-      <c r="O7" s="55"/>
-      <c r="P7" s="55"/>
-      <c r="Q7" s="55"/>
-      <c r="R7" s="55"/>
-      <c r="S7" s="55"/>
-      <c r="T7" s="55"/>
-      <c r="U7" s="55"/>
-      <c r="V7" s="55"/>
-      <c r="W7" s="55"/>
-      <c r="X7" s="55"/>
-      <c r="Y7" s="55"/>
-      <c r="Z7" s="55"/>
-      <c r="AA7" s="55"/>
-      <c r="AB7" s="60"/>
-      <c r="AC7" s="55"/>
-    </row>
-    <row r="8" spans="1:29" ht="10" customHeight="1">
-      <c r="A8" s="55"/>
-      <c r="B8" s="55"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
-      <c r="F8" s="55"/>
-      <c r="G8" s="61"/>
-      <c r="H8" s="55"/>
-      <c r="I8" s="61"/>
-      <c r="J8" s="61"/>
-      <c r="K8" s="61"/>
-      <c r="L8" s="55"/>
-      <c r="M8" s="102"/>
-      <c r="N8" s="55"/>
-      <c r="O8" s="102"/>
-      <c r="P8" s="61"/>
-      <c r="Q8" s="61"/>
-      <c r="R8" s="55"/>
-      <c r="S8" s="61"/>
-      <c r="T8" s="55"/>
-      <c r="U8" s="61"/>
-      <c r="V8" s="61"/>
-      <c r="W8" s="61"/>
-      <c r="X8" s="55"/>
-      <c r="Y8" s="61"/>
-      <c r="Z8" s="61"/>
-      <c r="AA8" s="61"/>
-      <c r="AB8" s="61"/>
-      <c r="AC8" s="55"/>
-    </row>
-    <row r="9" spans="1:29" ht="35" customHeight="1">
-      <c r="A9" s="57" t="s">
+      <c r="B9" s="27"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
+      <c r="F9" s="37"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="81"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="37"/>
+      <c r="L9" s="74"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="54"/>
+      <c r="P9" s="54"/>
+      <c r="Q9" s="82"/>
+      <c r="R9" s="30"/>
+      <c r="S9" s="30"/>
+      <c r="T9" s="29"/>
+      <c r="U9" s="37"/>
+      <c r="V9" s="37"/>
+      <c r="W9" s="37"/>
+      <c r="X9" s="37"/>
+      <c r="Y9" s="29"/>
+      <c r="Z9" s="30"/>
+      <c r="AA9" s="30"/>
+      <c r="AB9" s="30"/>
+      <c r="AC9" s="30"/>
+      <c r="AD9" s="31"/>
+    </row>
+    <row r="10" spans="1:30" ht="10.050000000000001" customHeight="1">
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="75"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="53"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="38"/>
+      <c r="R10" s="38"/>
+      <c r="S10" s="38"/>
+      <c r="T10" s="24"/>
+      <c r="U10" s="38"/>
+      <c r="V10" s="38"/>
+      <c r="W10" s="38"/>
+      <c r="X10" s="38"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="38"/>
+      <c r="AA10" s="38"/>
+      <c r="AB10" s="38"/>
+      <c r="AC10" s="38"/>
+      <c r="AD10" s="24"/>
+    </row>
+    <row r="11" spans="1:30" ht="19.95" customHeight="1">
+      <c r="A11" s="33" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="63"/>
-      <c r="C9" s="73"/>
-      <c r="D9" s="73"/>
-      <c r="E9" s="73"/>
-      <c r="F9" s="65"/>
-      <c r="G9" s="66"/>
-      <c r="H9" s="65"/>
-      <c r="I9" s="73"/>
-      <c r="J9" s="73"/>
-      <c r="K9" s="73"/>
-      <c r="L9" s="106"/>
-      <c r="M9" s="105"/>
-      <c r="N9" s="103"/>
-      <c r="O9" s="105"/>
-      <c r="P9" s="108"/>
-      <c r="Q9" s="73"/>
-      <c r="R9" s="65"/>
-      <c r="S9" s="66"/>
-      <c r="T9" s="65"/>
-      <c r="U9" s="73"/>
-      <c r="V9" s="73"/>
-      <c r="W9" s="73"/>
-      <c r="X9" s="65"/>
-      <c r="Y9" s="66"/>
-      <c r="Z9" s="66"/>
-      <c r="AA9" s="66"/>
-      <c r="AB9" s="66"/>
-      <c r="AC9" s="67"/>
-    </row>
-    <row r="10" spans="1:29" ht="10" customHeight="1">
-      <c r="A10" s="60"/>
-      <c r="B10" s="60"/>
-      <c r="C10" s="74"/>
-      <c r="D10" s="74"/>
-      <c r="E10" s="74"/>
-      <c r="F10" s="60"/>
-      <c r="G10" s="74"/>
-      <c r="H10" s="55"/>
-      <c r="I10" s="74"/>
-      <c r="J10" s="74"/>
-      <c r="K10" s="74"/>
-      <c r="L10" s="55"/>
-      <c r="M10" s="107"/>
-      <c r="N10" s="55"/>
-      <c r="O10" s="107"/>
-      <c r="P10" s="74"/>
-      <c r="Q10" s="74"/>
-      <c r="R10" s="60"/>
-      <c r="S10" s="74"/>
-      <c r="T10" s="60"/>
-      <c r="U10" s="74"/>
-      <c r="V10" s="74"/>
-      <c r="W10" s="74"/>
-      <c r="X10" s="55"/>
-      <c r="Y10" s="74"/>
-      <c r="Z10" s="74"/>
-      <c r="AA10" s="74"/>
-      <c r="AB10" s="74"/>
-      <c r="AC10" s="60"/>
-    </row>
-    <row r="11" spans="1:29" ht="20" customHeight="1">
-      <c r="A11" s="69" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="60"/>
-      <c r="C11" s="60"/>
-      <c r="D11" s="60"/>
-      <c r="E11" s="60"/>
-      <c r="F11" s="75"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="75"/>
-      <c r="K11" s="77" t="s">
-        <v>28</v>
-      </c>
-      <c r="L11" s="60"/>
-      <c r="M11" s="60"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="76"/>
-      <c r="P11" s="75"/>
-      <c r="Q11" s="77" t="s">
-        <v>29</v>
-      </c>
-      <c r="R11" s="75"/>
-      <c r="S11" s="60"/>
-      <c r="T11" s="60"/>
-      <c r="U11" s="75"/>
-      <c r="V11" s="75"/>
-      <c r="W11" s="75"/>
-      <c r="X11" s="75"/>
-      <c r="Y11" s="78" t="s">
-        <v>30</v>
-      </c>
-      <c r="Z11" s="55"/>
-      <c r="AA11" s="60"/>
-      <c r="AB11" s="60"/>
-      <c r="AC11" s="60"/>
-    </row>
-    <row r="12" spans="1:29" ht="10" customHeight="1">
-      <c r="A12" s="60"/>
-      <c r="B12" s="60"/>
-      <c r="C12" s="60"/>
-      <c r="D12" s="60"/>
-      <c r="E12" s="60"/>
-      <c r="F12" s="60"/>
-      <c r="G12" s="60"/>
-      <c r="H12" s="55"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-      <c r="K12" s="60"/>
-      <c r="L12" s="55"/>
-      <c r="M12" s="60"/>
-      <c r="N12" s="55"/>
-      <c r="O12" s="60"/>
-      <c r="P12" s="60"/>
-      <c r="Q12" s="60"/>
-      <c r="R12" s="60"/>
-      <c r="S12" s="60"/>
-      <c r="T12" s="60"/>
-      <c r="U12" s="60"/>
-      <c r="V12" s="60"/>
-      <c r="W12" s="60"/>
-      <c r="X12" s="55"/>
-      <c r="Y12" s="60"/>
-      <c r="Z12" s="60"/>
-      <c r="AA12" s="60"/>
-      <c r="AB12" s="60"/>
-      <c r="AC12" s="60"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="98"/>
+      <c r="G11" s="98"/>
+      <c r="H11" s="98"/>
+      <c r="I11" s="99"/>
+      <c r="J11" s="100"/>
+      <c r="K11" s="101"/>
+      <c r="L11" s="76"/>
+      <c r="M11" s="102"/>
+      <c r="N11" s="102"/>
+      <c r="O11" s="102"/>
+      <c r="P11" s="100"/>
+      <c r="Q11" s="103"/>
+      <c r="R11" s="101"/>
+      <c r="S11" s="102"/>
+      <c r="T11" s="102"/>
+      <c r="U11" s="100"/>
+      <c r="V11" s="100"/>
+      <c r="W11" s="103"/>
+      <c r="X11" s="100"/>
+      <c r="Y11" s="100"/>
+      <c r="Z11" s="104"/>
+      <c r="AA11" s="19"/>
+      <c r="AB11" s="24"/>
+      <c r="AC11" s="24"/>
+      <c r="AD11" s="24"/>
+    </row>
+    <row r="12" spans="1:30" ht="10.050000000000001" customHeight="1">
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="53"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="24"/>
+      <c r="L12" s="75"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="24"/>
+      <c r="Q12" s="53"/>
+      <c r="R12" s="24"/>
+      <c r="S12" s="24"/>
+      <c r="T12" s="24"/>
+      <c r="U12" s="24"/>
+      <c r="V12" s="24"/>
+      <c r="W12" s="53"/>
+      <c r="X12" s="24"/>
+      <c r="Y12" s="19"/>
+      <c r="Z12" s="24"/>
+      <c r="AA12" s="24"/>
+      <c r="AB12" s="24"/>
+      <c r="AC12" s="24"/>
+      <c r="AD12" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="AA1:AC1"/>
-    <mergeCell ref="AA2:AB2"/>
+    <mergeCell ref="AB1:AD1"/>
+    <mergeCell ref="AB2:AC2"/>
     <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="F1:H1"/>
     <mergeCell ref="K1:O1"/>
-    <mergeCell ref="P1:Z1"/>
+    <mergeCell ref="P1:AA1"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape"/>
@@ -3761,199 +3731,198 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="16.36328125" defaultRowHeight="18" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="16.33203125" defaultRowHeight="18" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="79" customWidth="1"/>
-    <col min="2" max="6" width="28.26953125" style="79" customWidth="1"/>
-    <col min="7" max="7" width="10" style="79" customWidth="1"/>
-    <col min="8" max="8" width="16.36328125" style="79" customWidth="1"/>
-    <col min="9" max="16384" width="16.36328125" style="79"/>
+    <col min="1" max="1" width="8.77734375" style="39" customWidth="1"/>
+    <col min="2" max="6" width="28.21875" style="39" customWidth="1"/>
+    <col min="7" max="7" width="10" style="39" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="39" customWidth="1"/>
+    <col min="9" max="16384" width="16.33203125" style="39"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="20.399999999999999" customHeight="1">
-      <c r="A1" s="80"/>
-      <c r="B1" s="81" t="s">
+      <c r="A1" s="40"/>
+      <c r="B1" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D1" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="F1" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="81" t="s">
+      <c r="G1" s="42"/>
+    </row>
+    <row r="2" spans="1:7" ht="20.399999999999999" customHeight="1">
+      <c r="A2" s="43"/>
+      <c r="B2" s="43"/>
+      <c r="C2" s="43"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+    </row>
+    <row r="3" spans="1:7" ht="24" customHeight="1">
+      <c r="A3" s="44">
+        <v>43106.447916666664</v>
+      </c>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="96"/>
+      <c r="F3" s="96"/>
+      <c r="G3" s="46">
+        <v>43106.447916666664</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="24" customHeight="1">
+      <c r="A4" s="47"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="96"/>
+      <c r="F4" s="96"/>
+      <c r="G4" s="48"/>
+    </row>
+    <row r="5" spans="1:7" ht="24" customHeight="1">
+      <c r="A5" s="47"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="96"/>
+      <c r="F5" s="96"/>
+      <c r="G5" s="48"/>
+    </row>
+    <row r="6" spans="1:7" ht="24" customHeight="1">
+      <c r="A6" s="47"/>
+      <c r="B6" s="45"/>
+      <c r="C6" s="45"/>
+      <c r="D6" s="45"/>
+      <c r="E6" s="96"/>
+      <c r="F6" s="96"/>
+      <c r="G6" s="48"/>
+    </row>
+    <row r="7" spans="1:7" ht="24" customHeight="1">
+      <c r="A7" s="47"/>
+      <c r="B7" s="45"/>
+      <c r="C7" s="45"/>
+      <c r="D7" s="45"/>
+      <c r="E7" s="96"/>
+      <c r="F7" s="96"/>
+      <c r="G7" s="48"/>
+    </row>
+    <row r="8" spans="1:7" ht="24" customHeight="1">
+      <c r="A8" s="47"/>
+      <c r="B8" s="45"/>
+      <c r="C8" s="45"/>
+      <c r="D8" s="45"/>
+      <c r="E8" s="96"/>
+      <c r="F8" s="96"/>
+      <c r="G8" s="48"/>
+    </row>
+    <row r="9" spans="1:7" ht="24" customHeight="1">
+      <c r="A9" s="44">
+        <v>43106.510416666664</v>
+      </c>
+      <c r="B9" s="95" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="81" t="s">
+      <c r="C9" s="96"/>
+      <c r="D9" s="95" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="81" t="s">
+      <c r="E9" s="97" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="81" t="s">
-        <v>36</v>
-      </c>
-      <c r="G1" s="82"/>
-    </row>
-    <row r="2" spans="1:7" ht="20.399999999999999" customHeight="1">
-      <c r="A2" s="83"/>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="83"/>
-    </row>
-    <row r="3" spans="1:7" ht="24" customHeight="1">
-      <c r="A3" s="84">
-        <v>43106.447916666664</v>
-      </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="98"/>
-      <c r="F3" s="98"/>
-      <c r="G3" s="86">
-        <v>43106.447916666664</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="24" customHeight="1">
-      <c r="A4" s="87"/>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="98"/>
-      <c r="F4" s="98"/>
-      <c r="G4" s="88"/>
-    </row>
-    <row r="5" spans="1:7" ht="24" customHeight="1">
-      <c r="A5" s="87"/>
-      <c r="B5" s="85"/>
-      <c r="C5" s="85"/>
-      <c r="D5" s="85"/>
-      <c r="E5" s="98"/>
-      <c r="F5" s="98"/>
-      <c r="G5" s="88"/>
-    </row>
-    <row r="6" spans="1:7" ht="24" customHeight="1">
-      <c r="A6" s="87"/>
-      <c r="B6" s="85"/>
-      <c r="C6" s="85"/>
-      <c r="D6" s="85"/>
-      <c r="E6" s="98"/>
-      <c r="F6" s="98"/>
-      <c r="G6" s="88"/>
-    </row>
-    <row r="7" spans="1:7" ht="24" customHeight="1">
-      <c r="A7" s="87"/>
-      <c r="B7" s="85"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="85"/>
-      <c r="E7" s="98"/>
-      <c r="F7" s="98"/>
-      <c r="G7" s="88"/>
-    </row>
-    <row r="8" spans="1:7" ht="24" customHeight="1">
-      <c r="A8" s="87"/>
-      <c r="B8" s="85"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="85"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="88"/>
-    </row>
-    <row r="9" spans="1:7" ht="24" customHeight="1">
-      <c r="A9" s="84">
+      <c r="F9" s="96"/>
+      <c r="G9" s="46">
         <v>43106.510416666664</v>
       </c>
-      <c r="B9" s="99" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="98"/>
-      <c r="D9" s="99" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="100" t="s">
-        <v>39</v>
-      </c>
-      <c r="F9" s="98"/>
-      <c r="G9" s="86">
-        <v>43106.510416666664</v>
-      </c>
     </row>
     <row r="10" spans="1:7" ht="24" customHeight="1">
-      <c r="A10" s="87"/>
-      <c r="B10" s="98"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="98"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="88"/>
+      <c r="A10" s="47"/>
+      <c r="B10" s="96"/>
+      <c r="C10" s="96"/>
+      <c r="D10" s="96"/>
+      <c r="E10" s="96"/>
+      <c r="F10" s="96"/>
+      <c r="G10" s="48"/>
     </row>
     <row r="11" spans="1:7" ht="24" customHeight="1">
-      <c r="A11" s="87"/>
-      <c r="B11" s="98"/>
-      <c r="C11" s="98"/>
-      <c r="D11" s="98"/>
-      <c r="E11" s="98"/>
-      <c r="F11" s="98"/>
-      <c r="G11" s="88"/>
+      <c r="A11" s="47"/>
+      <c r="B11" s="96"/>
+      <c r="C11" s="96"/>
+      <c r="D11" s="96"/>
+      <c r="E11" s="96"/>
+      <c r="F11" s="96"/>
+      <c r="G11" s="48"/>
     </row>
     <row r="12" spans="1:7" ht="24" customHeight="1">
-      <c r="A12" s="87"/>
-      <c r="B12" s="98"/>
-      <c r="C12" s="98"/>
-      <c r="D12" s="98"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="88"/>
+      <c r="A12" s="47"/>
+      <c r="B12" s="96"/>
+      <c r="C12" s="96"/>
+      <c r="D12" s="96"/>
+      <c r="E12" s="96"/>
+      <c r="F12" s="96"/>
+      <c r="G12" s="48"/>
     </row>
     <row r="13" spans="1:7" ht="24" customHeight="1">
-      <c r="A13" s="87"/>
-      <c r="B13" s="98"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="98"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="98"/>
-      <c r="G13" s="88"/>
+      <c r="A13" s="47"/>
+      <c r="B13" s="96"/>
+      <c r="C13" s="96"/>
+      <c r="D13" s="96"/>
+      <c r="E13" s="96"/>
+      <c r="F13" s="96"/>
+      <c r="G13" s="48"/>
     </row>
     <row r="14" spans="1:7" ht="24" customHeight="1">
-      <c r="A14" s="87"/>
-      <c r="B14" s="98"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="98"/>
-      <c r="E14" s="98"/>
-      <c r="F14" s="98"/>
-      <c r="G14" s="88"/>
+      <c r="A14" s="47"/>
+      <c r="B14" s="96"/>
+      <c r="C14" s="96"/>
+      <c r="D14" s="96"/>
+      <c r="E14" s="96"/>
+      <c r="F14" s="96"/>
+      <c r="G14" s="48"/>
     </row>
     <row r="15" spans="1:7" ht="24" customHeight="1">
-      <c r="A15" s="84">
+      <c r="A15" s="44">
         <v>43111.083333333336</v>
       </c>
-      <c r="B15" s="98"/>
-      <c r="C15" s="98"/>
-      <c r="D15" s="98"/>
-      <c r="E15" s="98"/>
-      <c r="F15" s="98"/>
-      <c r="G15" s="86">
+      <c r="B15" s="96"/>
+      <c r="C15" s="96"/>
+      <c r="D15" s="96"/>
+      <c r="E15" s="96"/>
+      <c r="F15" s="96"/>
+      <c r="G15" s="46">
         <v>43106.572916666664</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="24" customHeight="1">
-      <c r="A16" s="87"/>
-      <c r="B16" s="85"/>
-      <c r="C16" s="98"/>
-      <c r="D16" s="85"/>
-      <c r="E16" s="85"/>
-      <c r="F16" s="98"/>
-      <c r="G16" s="88"/>
+      <c r="A16" s="47"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="96"/>
+      <c r="D16" s="45"/>
+      <c r="E16" s="45"/>
+      <c r="F16" s="96"/>
+      <c r="G16" s="48"/>
     </row>
     <row r="17" spans="1:7" ht="24" customHeight="1">
-      <c r="A17" s="87"/>
-      <c r="B17" s="85"/>
-      <c r="C17" s="98"/>
-      <c r="D17" s="85"/>
-      <c r="E17" s="85"/>
-      <c r="F17" s="98"/>
-      <c r="G17" s="88"/>
+      <c r="A17" s="47"/>
+      <c r="B17" s="45"/>
+      <c r="C17" s="96"/>
+      <c r="D17" s="45"/>
+      <c r="E17" s="45"/>
+      <c r="F17" s="96"/>
+      <c r="G17" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="E3:E8"/>
     <mergeCell ref="F3:F8"/>
     <mergeCell ref="F9:F14"/>
     <mergeCell ref="F15:F17"/>
@@ -3962,6 +3931,7 @@
     <mergeCell ref="C15:C17"/>
     <mergeCell ref="D9:D15"/>
     <mergeCell ref="E9:E15"/>
+    <mergeCell ref="E3:E8"/>
   </mergeCells>
   <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
   <pageSetup orientation="landscape"/>

</xml_diff>